<commit_message>
Align D7 regimes and aggregation readiness
</commit_message>
<xml_diff>
--- a/Project 1 Data Quality Assessment/D7 Topological Role Consistency and Structural Representativeness/outputs/local/D7_ablation_redundancy.xlsx
+++ b/Project 1 Data Quality Assessment/D7 Topological Role Consistency and Structural Representativeness/outputs/local/D7_ablation_redundancy.xlsx
@@ -495,10 +495,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.9088378379444186</v>
+        <v>0.9093318699981358</v>
       </c>
       <c r="C3" t="n">
-        <v>0.8719191778273809</v>
+        <v>0.8625023251488095</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -513,10 +513,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.9319975265451969</v>
+        <v>0.9335896422851648</v>
       </c>
       <c r="C4" t="n">
-        <v>0.8966936383928571</v>
+        <v>0.8804059709821429</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -531,10 +531,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.9869100341751171</v>
+        <v>0.9872713198864503</v>
       </c>
       <c r="C5" t="n">
-        <v>0.9137718563988095</v>
+        <v>0.9088192894345238</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -549,10 +549,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.8915406236721906</v>
+        <v>0.8774729642396752</v>
       </c>
       <c r="C6" t="n">
-        <v>0.8576195126488095</v>
+        <v>0.8463774181547619</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -604,7 +604,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="23" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
   </cols>
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.04332128706688192</v>
+        <v>0.04817068966358561</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -656,7 +656,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.8389483742925048</v>
+        <v>0.8251274138495348</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -674,7 +674,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.9791724436804865</v>
+        <v>0.9619507138943536</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -692,7 +692,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-0.004124947116062594</v>
+        <v>-0.01158745828044938</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -719,7 +719,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
     <col width="38" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
@@ -747,7 +747,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.08787031315444654</v>
+        <v>0.1072949580849036</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -762,7 +762,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.02573950503666441</v>
+        <v>0.02021875233732925</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -777,7 +777,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.1023486350905899</v>
+        <v>0.05961396256854015</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Reclassify D7 topology evidence and gates
</commit_message>
<xml_diff>
--- a/Project 1 Data Quality Assessment/D7 Topological Role Consistency and Structural Representativeness/outputs/local/D7_ablation_redundancy.xlsx
+++ b/Project 1 Data Quality Assessment/D7 Topological Role Consistency and Structural Representativeness/outputs/local/D7_ablation_redundancy.xlsx
@@ -943,7 +943,7 @@
   <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="39" customWidth="1" min="1" max="1"/>
     <col width="36" customWidth="1" min="2" max="2"/>
     <col width="45" customWidth="1" min="3" max="3"/>
   </cols>
@@ -968,7 +968,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>topology_not_field_verified</t>
+          <t>production_topology_not_dual_approved</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -978,7 +978,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>verify drawing asset serial channel position and obtain two approvals</t>
+          <t>audit documentary evidence and maintenance history, then obtain two approvals</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Finalize D7 scientific aggregation readiness
</commit_message>
<xml_diff>
--- a/Project 1 Data Quality Assessment/D7 Topological Role Consistency and Structural Representativeness/outputs/local/D7_ablation_redundancy.xlsx
+++ b/Project 1 Data Quality Assessment/D7 Topological Role Consistency and Structural Representativeness/outputs/local/D7_ablation_redundancy.xlsx
@@ -22,7 +22,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'partial_correlation'!$A$1:$A$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'vif_mutual_information'!$A$1:$A$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'d6_handshake'!$A$1:$F$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'failure_cases'!$A$1:$C$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'failure_cases'!$A$1:$C$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -800,7 +800,7 @@
   <dimension ref="A1:A2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -813,7 +813,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>not_claimed_before_verified_topology_and_external_labels</t>
+          <t>planned_for_final_WW_DQS_overlap_audit</t>
         </is>
       </c>
     </row>
@@ -869,7 +869,7 @@
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="36" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -907,7 +907,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>d7-d6-v2.1</t>
+          <t>d7-d6-v2.2</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -919,12 +919,10 @@
       <c r="D2" t="n">
         <v>0</v>
       </c>
-      <c r="E2" t="n">
-        <v>0</v>
-      </c>
+      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>no_D6_write_path_static_isolation_pass</t>
+          <t>non_destructive_arbitration_runs_after_validation</t>
         </is>
       </c>
     </row>
@@ -940,11 +938,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39" customWidth="1" min="1" max="1"/>
-    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
     <col width="45" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
@@ -968,17 +966,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>production_topology_not_dual_approved</t>
+          <t>deployment_topology_not_dual_approved</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>D7_total_and_D7_forDQR_null</t>
+          <t>automated_control_release_blocked</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>audit documentary evidence and maintenance history, then obtain two approvals</t>
+          <t>retain offline scientific score and block only automated deployment</t>
         </is>
       </c>
     </row>
@@ -990,17 +988,34 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>most templates cannot gate or veto</t>
+          <t>L1 templates remain diagnostic and cannot trigger action</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>collect qualified multi-season blocks and pass external validation</t>
+          <t>use validation-graded L2/L3 admission and report coverage explicitly</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>node_localization_below_target</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>sensor-specific hard Veto disabled</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>retain process-coherence protection and report node attribution as evidence only</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C3"/>
+  <autoFilter ref="A1:C4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Finalize D7 hierarchical admission and dual interfaces
</commit_message>
<xml_diff>
--- a/Project 1 Data Quality Assessment/D7 Topological Role Consistency and Structural Representativeness/outputs/local/D7_ablation_redundancy.xlsx
+++ b/Project 1 Data Quality Assessment/D7 Topological Role Consistency and Structural Representativeness/outputs/local/D7_ablation_redundancy.xlsx
@@ -907,7 +907,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>d7-d6-v2.2</t>
+          <t>d7-d6-v2.3</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -1010,7 +1010,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>retain process-coherence protection and report node attribution as evidence only</t>
+          <t>retain the process-coherence attribution guard and report node attribution as evidence only</t>
         </is>
       </c>
     </row>

</xml_diff>